<commit_message>
Align the xlsx Summary sheet with inherited-parts-explained.md
Same 8 rows, same explanations (condensed for a cell) -- the 'What we
actually borrow' column now carries the plain-language mechanism explanation
instead of a one-phrase label, so the spreadsheet and the markdown doc say
the same thing at matching detail. Widened that column and added row heights
for readability.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full detail'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -487,14 +487,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,15 +524,15 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>0. Data</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>50Salads video + its transcript; no frame timestamps at any point</t>
+          <t>Raw video + ordered transcript, no timestamps anywhere</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -542,30 +542,30 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Task definition and weak-supervision constraint</t>
+          <t>The weak-supervision setup itself, not a technique: only the ordered list of actions is ever given, never when each one starts or ends. Everything downstream has to work under that constraint.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
     </row>
-    <row r="3">
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1. Similarity</t>
+          <t>Semantic front-end</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Cosine-match each transcript action's text embedding against every frame</t>
+          <t>Encode short video clips and transcript actions into a shared semantic space</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>OVTAS (FAES)</t>
+          <t>OVTAS</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Zero-shot VLM matching, scored per transcript position rather than open-vocab</t>
+          <t>Score a frame against an action using a frozen vision-language model, with no training: encode the frame and the action label into the same space and take cosine similarity. OVTAS scores against an open, unordered action list; we score against the actions in the order the transcript gives them.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -574,25 +574,25 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2. Coarse decode</t>
+          <t>Stage A: coarse alignment</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Turn that similarity into one ordered, monotone segmentation of the whole video</t>
+          <t>Build the cost and force actions to appear in transcript order</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>ASOT solver + HiERO-StepG's monotonicity constraint</t>
+          <t>HiERO-StepG (+ our own dynamic programming)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>`delta.align.asot`: fused-GW OT with a transcript-order prior, so a weak signal still degrades to something sane</t>
+          <t>Force the predicted timeline to respect the transcript's order with no exceptions -- if action 3 comes after action 2 in the recipe, its segment must come after action 2's in time, always. Done algorithmically (DP/OT), not learned, which rules out most wrong placements before the visual match matters.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -601,48 +601,52 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="75" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>3. Per-boundary search</t>
+          <t>Stage B1: segment extent</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Slide a window across each coarse cut and score every candidate split point</t>
+          <t>Find the confident temporal extent of each action around its coarse location</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>designed for this project</t>
+          <t>HiERO-StepG</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>`delta.align.refine`: scores + a prominence confidence per boundary</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
+          <t>Once you have a rough position, look at a local window around it to refine it -- check frames just before/after the rough boundary and ask whether they still belong to that action, rather than trusting the coarse placement as final.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.31227</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="105" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>4. Confidence-gated training signal</t>
+          <t>Stage B2: exact transition</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Only the boundaries the search trusts become training anchors</t>
+          <t>Search specifically for the best crossover point</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>CVA's boundary-contrastive idea, MASRA's relational loss</t>
+          <t>our design, inspired by CVA + MASRA</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>`delta.align.cbd` (PBCR) + `delta.align.masra_torch`: rebuilt on our own confident boundaries, not GT spans</t>
+          <t>Two principles, not reused code: from CVA, a boundary frame should look the same regardless of context and be distinct from its neighbours (CVA anchors this on GT boundaries, which we don't have). From MASRA, judge frames by how they relate to each other, not in isolation, and match that structure to what the transcript implies. Rebuilt on our own confident current guess, not GT.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -651,118 +655,89 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="90" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>5. Encoder</t>
+          <t>Optional Stage C</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>One frozen model behind steps 1-4</t>
+          <t>Improve frame / segment consistency if boundaries remain noisy</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>VideoLLaMA3</t>
+          <t>CLOT / D-CLOT</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Similarity embeddings + captioning/reasoning from a single family, per the supervisor's direction</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2501.13106</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Alternate between refining frame-level detail and segment-level structure repeatedly, each informing the other. D-CLOT adds: periodically re-check whether each action's 'typical example' is still accurate, especially for short or easily-confused actions. A fallback, only if earlier stages aren't enough.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf ; https://arxiv.org/abs/2608.05877</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>6. Fallback if noisy</t>
+          <t>Optional Stage D</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Re-estimate segment prototypes when short/ambiguous actions keep failing</t>
+          <t>Reason only about difficult boundaries</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>CLOT / D-CLOT</t>
+          <t>TOGA / VideoLLaMA3</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Only triggered if step 4 isn't enough</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2608.05877</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>Ask a language-capable video model directly, but only when cheaper methods are unsure. TOGA gets a VLM to answer 'when does this happen?' with no GT timestamps by checking self-consistency (its answer, asked back as a question, should describe the same event). Expensive -- only for the lowest-confidence boundaries.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2506.09445 ; https://arxiv.org/abs/2501.13106</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="75" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>7. Fallback for hard cases</t>
+          <t>Output</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Spend an expensive chat-VLM call only on the lowest-confidence boundaries</t>
+          <t>Convert refined boundaries into dense Y*</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>TOGA</t>
+          <t>DELTA</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Selective, not run on every frame</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2506.09445</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>8. Interface out</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Dense per-frame labels handed to the unchanged DELTA decoder</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>DELTA</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>No change to anything downstream</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
+          <t>The format everything must be handed back in: one label per video frame, because that's what DELTA's existing downstream anticipation model expects. We don't change that interface, only what produces the labels feeding into it.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:E9"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>